<commit_message>
chore: update dashboard data
</commit_message>
<xml_diff>
--- a/Master_Data.xlsx
+++ b/Master_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dashboard_Bakso Ibu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4FA6FB-3E36-440C-8D45-0946677D49C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92982881-9AFB-4865-8D28-D5B90FE1D1F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4584C4D0-F1D3-4CAB-AEE3-EEE67B00564C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2247" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2666" uniqueCount="125">
   <si>
     <t>product</t>
   </si>
@@ -402,6 +402,15 @@
   </si>
   <si>
     <t>KERUPUK PANGSIT ISI</t>
+  </si>
+  <si>
+    <t>Juni</t>
+  </si>
+  <si>
+    <t>BAKSO MOZA SATUAN</t>
+  </si>
+  <si>
+    <t>CAMPUR</t>
   </si>
 </sst>
 </file>
@@ -780,7 +789,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A6087EF-6223-49E4-BB6C-DBD7179421B2}">
-  <dimension ref="A1:S441"/>
+  <dimension ref="A1:S524"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
@@ -20307,6 +20316,3670 @@
         <v>88</v>
       </c>
     </row>
+    <row r="442" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A442" t="s">
+        <v>19</v>
+      </c>
+      <c r="D442" t="s">
+        <v>20</v>
+      </c>
+      <c r="H442">
+        <v>609</v>
+      </c>
+      <c r="I442" t="s">
+        <v>21</v>
+      </c>
+      <c r="J442">
+        <v>3564500</v>
+      </c>
+      <c r="K442">
+        <v>0</v>
+      </c>
+      <c r="L442">
+        <v>0</v>
+      </c>
+      <c r="M442">
+        <v>3564500</v>
+      </c>
+      <c r="N442">
+        <v>0</v>
+      </c>
+      <c r="O442">
+        <v>3564500</v>
+      </c>
+      <c r="P442">
+        <v>468</v>
+      </c>
+      <c r="Q442">
+        <v>1.3</v>
+      </c>
+      <c r="R442" t="s">
+        <v>122</v>
+      </c>
+      <c r="S442" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="443" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A443" t="s">
+        <v>24</v>
+      </c>
+      <c r="D443" t="s">
+        <v>25</v>
+      </c>
+      <c r="H443">
+        <v>195</v>
+      </c>
+      <c r="I443" t="s">
+        <v>21</v>
+      </c>
+      <c r="J443">
+        <v>6240000</v>
+      </c>
+      <c r="K443">
+        <v>0</v>
+      </c>
+      <c r="L443">
+        <v>0</v>
+      </c>
+      <c r="M443">
+        <v>6240000</v>
+      </c>
+      <c r="N443">
+        <v>0</v>
+      </c>
+      <c r="O443">
+        <v>6240000</v>
+      </c>
+      <c r="P443">
+        <v>181</v>
+      </c>
+      <c r="Q443">
+        <v>1.08</v>
+      </c>
+      <c r="R443" t="s">
+        <v>122</v>
+      </c>
+      <c r="S443" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="444" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A444" t="s">
+        <v>27</v>
+      </c>
+      <c r="D444" t="s">
+        <v>25</v>
+      </c>
+      <c r="H444">
+        <v>608</v>
+      </c>
+      <c r="I444" t="s">
+        <v>21</v>
+      </c>
+      <c r="J444">
+        <v>15200000</v>
+      </c>
+      <c r="K444">
+        <v>0</v>
+      </c>
+      <c r="L444">
+        <v>0</v>
+      </c>
+      <c r="M444">
+        <v>15200000</v>
+      </c>
+      <c r="N444">
+        <v>0</v>
+      </c>
+      <c r="O444">
+        <v>15200000</v>
+      </c>
+      <c r="P444">
+        <v>449</v>
+      </c>
+      <c r="Q444">
+        <v>1.35</v>
+      </c>
+      <c r="R444" t="s">
+        <v>122</v>
+      </c>
+      <c r="S444" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="445" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A445" t="s">
+        <v>28</v>
+      </c>
+      <c r="D445" t="s">
+        <v>25</v>
+      </c>
+      <c r="H445">
+        <v>561</v>
+      </c>
+      <c r="I445" t="s">
+        <v>21</v>
+      </c>
+      <c r="J445">
+        <v>10082000</v>
+      </c>
+      <c r="K445">
+        <v>0</v>
+      </c>
+      <c r="L445">
+        <v>0</v>
+      </c>
+      <c r="M445">
+        <v>10082000</v>
+      </c>
+      <c r="N445">
+        <v>0</v>
+      </c>
+      <c r="O445">
+        <v>10082000</v>
+      </c>
+      <c r="P445">
+        <v>421</v>
+      </c>
+      <c r="Q445">
+        <v>1.33</v>
+      </c>
+      <c r="R445" t="s">
+        <v>122</v>
+      </c>
+      <c r="S445" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="446" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A446" t="s">
+        <v>29</v>
+      </c>
+      <c r="D446" t="s">
+        <v>25</v>
+      </c>
+      <c r="H446">
+        <v>1</v>
+      </c>
+      <c r="I446" t="s">
+        <v>21</v>
+      </c>
+      <c r="J446">
+        <v>20000</v>
+      </c>
+      <c r="K446">
+        <v>0</v>
+      </c>
+      <c r="L446">
+        <v>0</v>
+      </c>
+      <c r="M446">
+        <v>20000</v>
+      </c>
+      <c r="N446">
+        <v>0</v>
+      </c>
+      <c r="O446">
+        <v>20000</v>
+      </c>
+      <c r="P446">
+        <v>1</v>
+      </c>
+      <c r="Q446">
+        <v>1</v>
+      </c>
+      <c r="R446" t="s">
+        <v>122</v>
+      </c>
+      <c r="S446" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="447" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A447" t="s">
+        <v>30</v>
+      </c>
+      <c r="D447" t="s">
+        <v>25</v>
+      </c>
+      <c r="H447">
+        <v>287</v>
+      </c>
+      <c r="I447" t="s">
+        <v>21</v>
+      </c>
+      <c r="J447">
+        <v>5738000</v>
+      </c>
+      <c r="K447">
+        <v>0</v>
+      </c>
+      <c r="L447">
+        <v>0</v>
+      </c>
+      <c r="M447">
+        <v>5738000</v>
+      </c>
+      <c r="N447">
+        <v>0</v>
+      </c>
+      <c r="O447">
+        <v>5738000</v>
+      </c>
+      <c r="P447">
+        <v>257</v>
+      </c>
+      <c r="Q447">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="R447" t="s">
+        <v>122</v>
+      </c>
+      <c r="S447" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="448" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A448" t="s">
+        <v>31</v>
+      </c>
+      <c r="D448" t="s">
+        <v>25</v>
+      </c>
+      <c r="H448">
+        <v>1093</v>
+      </c>
+      <c r="I448" t="s">
+        <v>21</v>
+      </c>
+      <c r="J448">
+        <v>32769000</v>
+      </c>
+      <c r="K448">
+        <v>0</v>
+      </c>
+      <c r="L448">
+        <v>0</v>
+      </c>
+      <c r="M448">
+        <v>32769000</v>
+      </c>
+      <c r="N448">
+        <v>0</v>
+      </c>
+      <c r="O448">
+        <v>32769000</v>
+      </c>
+      <c r="P448">
+        <v>828</v>
+      </c>
+      <c r="Q448">
+        <v>1.32</v>
+      </c>
+      <c r="R448" t="s">
+        <v>122</v>
+      </c>
+      <c r="S448" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="449" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A449" t="s">
+        <v>33</v>
+      </c>
+      <c r="D449" t="s">
+        <v>25</v>
+      </c>
+      <c r="H449">
+        <v>388</v>
+      </c>
+      <c r="I449" t="s">
+        <v>21</v>
+      </c>
+      <c r="J449">
+        <v>8924000</v>
+      </c>
+      <c r="K449">
+        <v>0</v>
+      </c>
+      <c r="L449">
+        <v>0</v>
+      </c>
+      <c r="M449">
+        <v>8924000</v>
+      </c>
+      <c r="N449">
+        <v>0</v>
+      </c>
+      <c r="O449">
+        <v>8924000</v>
+      </c>
+      <c r="P449">
+        <v>323</v>
+      </c>
+      <c r="Q449">
+        <v>1.2</v>
+      </c>
+      <c r="R449" t="s">
+        <v>122</v>
+      </c>
+      <c r="S449" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="450" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A450" t="s">
+        <v>35</v>
+      </c>
+      <c r="D450" t="s">
+        <v>25</v>
+      </c>
+      <c r="H450">
+        <v>1056</v>
+      </c>
+      <c r="I450" t="s">
+        <v>21</v>
+      </c>
+      <c r="J450">
+        <v>21108000</v>
+      </c>
+      <c r="K450">
+        <v>0</v>
+      </c>
+      <c r="L450">
+        <v>0</v>
+      </c>
+      <c r="M450">
+        <v>21108000</v>
+      </c>
+      <c r="N450">
+        <v>0</v>
+      </c>
+      <c r="O450">
+        <v>21108000</v>
+      </c>
+      <c r="P450">
+        <v>765</v>
+      </c>
+      <c r="Q450">
+        <v>1.38</v>
+      </c>
+      <c r="R450" t="s">
+        <v>122</v>
+      </c>
+      <c r="S450" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="451" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A451" t="s">
+        <v>36</v>
+      </c>
+      <c r="D451" t="s">
+        <v>25</v>
+      </c>
+      <c r="H451">
+        <v>843</v>
+      </c>
+      <c r="I451" t="s">
+        <v>21</v>
+      </c>
+      <c r="J451">
+        <v>21075000</v>
+      </c>
+      <c r="K451">
+        <v>0</v>
+      </c>
+      <c r="L451">
+        <v>0</v>
+      </c>
+      <c r="M451">
+        <v>21075000</v>
+      </c>
+      <c r="N451">
+        <v>0</v>
+      </c>
+      <c r="O451">
+        <v>21075000</v>
+      </c>
+      <c r="P451">
+        <v>626</v>
+      </c>
+      <c r="Q451">
+        <v>1.35</v>
+      </c>
+      <c r="R451" t="s">
+        <v>122</v>
+      </c>
+      <c r="S451" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="452" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A452" t="s">
+        <v>39</v>
+      </c>
+      <c r="D452" t="s">
+        <v>25</v>
+      </c>
+      <c r="H452">
+        <v>1</v>
+      </c>
+      <c r="I452" t="s">
+        <v>21</v>
+      </c>
+      <c r="J452">
+        <v>23000</v>
+      </c>
+      <c r="K452">
+        <v>0</v>
+      </c>
+      <c r="L452">
+        <v>0</v>
+      </c>
+      <c r="M452">
+        <v>23000</v>
+      </c>
+      <c r="N452">
+        <v>0</v>
+      </c>
+      <c r="O452">
+        <v>23000</v>
+      </c>
+      <c r="P452">
+        <v>1</v>
+      </c>
+      <c r="Q452">
+        <v>1</v>
+      </c>
+      <c r="R452" t="s">
+        <v>122</v>
+      </c>
+      <c r="S452" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="453" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A453" t="s">
+        <v>40</v>
+      </c>
+      <c r="D453" t="s">
+        <v>25</v>
+      </c>
+      <c r="H453">
+        <v>1</v>
+      </c>
+      <c r="I453" t="s">
+        <v>21</v>
+      </c>
+      <c r="J453">
+        <v>25000</v>
+      </c>
+      <c r="K453">
+        <v>0</v>
+      </c>
+      <c r="L453">
+        <v>0</v>
+      </c>
+      <c r="M453">
+        <v>25000</v>
+      </c>
+      <c r="N453">
+        <v>0</v>
+      </c>
+      <c r="O453">
+        <v>25000</v>
+      </c>
+      <c r="P453">
+        <v>1</v>
+      </c>
+      <c r="Q453">
+        <v>1</v>
+      </c>
+      <c r="R453" t="s">
+        <v>122</v>
+      </c>
+      <c r="S453" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="454" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A454" t="s">
+        <v>43</v>
+      </c>
+      <c r="D454" t="s">
+        <v>44</v>
+      </c>
+      <c r="H454">
+        <v>778</v>
+      </c>
+      <c r="I454" t="s">
+        <v>21</v>
+      </c>
+      <c r="J454">
+        <v>3890000</v>
+      </c>
+      <c r="K454">
+        <v>0</v>
+      </c>
+      <c r="L454">
+        <v>0</v>
+      </c>
+      <c r="M454">
+        <v>3890000</v>
+      </c>
+      <c r="N454">
+        <v>0</v>
+      </c>
+      <c r="O454">
+        <v>3890000</v>
+      </c>
+      <c r="P454">
+        <v>640</v>
+      </c>
+      <c r="Q454">
+        <v>1.22</v>
+      </c>
+      <c r="R454" t="s">
+        <v>122</v>
+      </c>
+      <c r="S454" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="455" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A455" t="s">
+        <v>46</v>
+      </c>
+      <c r="D455" t="s">
+        <v>44</v>
+      </c>
+      <c r="H455">
+        <v>35</v>
+      </c>
+      <c r="I455" t="s">
+        <v>21</v>
+      </c>
+      <c r="J455">
+        <v>595000</v>
+      </c>
+      <c r="K455">
+        <v>0</v>
+      </c>
+      <c r="L455">
+        <v>0</v>
+      </c>
+      <c r="M455">
+        <v>595000</v>
+      </c>
+      <c r="N455">
+        <v>0</v>
+      </c>
+      <c r="O455">
+        <v>595000</v>
+      </c>
+      <c r="P455">
+        <v>29</v>
+      </c>
+      <c r="Q455">
+        <v>1.21</v>
+      </c>
+      <c r="R455" t="s">
+        <v>122</v>
+      </c>
+      <c r="S455" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="456" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A456" t="s">
+        <v>47</v>
+      </c>
+      <c r="D456" t="s">
+        <v>44</v>
+      </c>
+      <c r="H456">
+        <v>55</v>
+      </c>
+      <c r="I456" t="s">
+        <v>21</v>
+      </c>
+      <c r="J456">
+        <v>275000</v>
+      </c>
+      <c r="K456">
+        <v>0</v>
+      </c>
+      <c r="L456">
+        <v>0</v>
+      </c>
+      <c r="M456">
+        <v>275000</v>
+      </c>
+      <c r="N456">
+        <v>0</v>
+      </c>
+      <c r="O456">
+        <v>275000</v>
+      </c>
+      <c r="P456">
+        <v>46</v>
+      </c>
+      <c r="Q456">
+        <v>1.2</v>
+      </c>
+      <c r="R456" t="s">
+        <v>122</v>
+      </c>
+      <c r="S456" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="457" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A457" t="s">
+        <v>49</v>
+      </c>
+      <c r="D457" t="s">
+        <v>50</v>
+      </c>
+      <c r="H457">
+        <v>29</v>
+      </c>
+      <c r="I457" t="s">
+        <v>21</v>
+      </c>
+      <c r="J457">
+        <v>522000</v>
+      </c>
+      <c r="K457">
+        <v>0</v>
+      </c>
+      <c r="L457">
+        <v>0</v>
+      </c>
+      <c r="M457">
+        <v>522000</v>
+      </c>
+      <c r="N457">
+        <v>0</v>
+      </c>
+      <c r="O457">
+        <v>522000</v>
+      </c>
+      <c r="P457">
+        <v>26</v>
+      </c>
+      <c r="Q457">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="R457" t="s">
+        <v>122</v>
+      </c>
+      <c r="S457" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="458" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A458" t="s">
+        <v>51</v>
+      </c>
+      <c r="D458" t="s">
+        <v>50</v>
+      </c>
+      <c r="H458">
+        <v>8</v>
+      </c>
+      <c r="I458" t="s">
+        <v>21</v>
+      </c>
+      <c r="J458">
+        <v>20000</v>
+      </c>
+      <c r="K458">
+        <v>0</v>
+      </c>
+      <c r="L458">
+        <v>0</v>
+      </c>
+      <c r="M458">
+        <v>20000</v>
+      </c>
+      <c r="N458">
+        <v>0</v>
+      </c>
+      <c r="O458">
+        <v>20000</v>
+      </c>
+      <c r="P458">
+        <v>4</v>
+      </c>
+      <c r="Q458">
+        <v>2</v>
+      </c>
+      <c r="R458" t="s">
+        <v>122</v>
+      </c>
+      <c r="S458" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="459" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A459" t="s">
+        <v>52</v>
+      </c>
+      <c r="D459" t="s">
+        <v>50</v>
+      </c>
+      <c r="H459">
+        <v>5</v>
+      </c>
+      <c r="I459" t="s">
+        <v>21</v>
+      </c>
+      <c r="J459">
+        <v>12500</v>
+      </c>
+      <c r="K459">
+        <v>0</v>
+      </c>
+      <c r="L459">
+        <v>0</v>
+      </c>
+      <c r="M459">
+        <v>12500</v>
+      </c>
+      <c r="N459">
+        <v>0</v>
+      </c>
+      <c r="O459">
+        <v>12500</v>
+      </c>
+      <c r="P459">
+        <v>4</v>
+      </c>
+      <c r="Q459">
+        <v>1.25</v>
+      </c>
+      <c r="R459" t="s">
+        <v>122</v>
+      </c>
+      <c r="S459" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="460" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A460" t="s">
+        <v>53</v>
+      </c>
+      <c r="D460" t="s">
+        <v>50</v>
+      </c>
+      <c r="H460">
+        <v>7</v>
+      </c>
+      <c r="I460" t="s">
+        <v>21</v>
+      </c>
+      <c r="J460">
+        <v>105000</v>
+      </c>
+      <c r="K460">
+        <v>0</v>
+      </c>
+      <c r="L460">
+        <v>0</v>
+      </c>
+      <c r="M460">
+        <v>105000</v>
+      </c>
+      <c r="N460">
+        <v>0</v>
+      </c>
+      <c r="O460">
+        <v>105000</v>
+      </c>
+      <c r="P460">
+        <v>6</v>
+      </c>
+      <c r="Q460">
+        <v>1.17</v>
+      </c>
+      <c r="R460" t="s">
+        <v>122</v>
+      </c>
+      <c r="S460" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="461" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A461" t="s">
+        <v>123</v>
+      </c>
+      <c r="D461" t="s">
+        <v>50</v>
+      </c>
+      <c r="H461">
+        <v>1</v>
+      </c>
+      <c r="I461" t="s">
+        <v>21</v>
+      </c>
+      <c r="J461">
+        <v>15000</v>
+      </c>
+      <c r="K461">
+        <v>0</v>
+      </c>
+      <c r="L461">
+        <v>0</v>
+      </c>
+      <c r="M461">
+        <v>15000</v>
+      </c>
+      <c r="N461">
+        <v>0</v>
+      </c>
+      <c r="O461">
+        <v>15000</v>
+      </c>
+      <c r="P461">
+        <v>1</v>
+      </c>
+      <c r="Q461">
+        <v>1</v>
+      </c>
+      <c r="R461" t="s">
+        <v>122</v>
+      </c>
+      <c r="S461" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="462" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A462" t="s">
+        <v>54</v>
+      </c>
+      <c r="D462" t="s">
+        <v>50</v>
+      </c>
+      <c r="H462">
+        <v>6</v>
+      </c>
+      <c r="I462" t="s">
+        <v>21</v>
+      </c>
+      <c r="J462">
+        <v>30000</v>
+      </c>
+      <c r="K462">
+        <v>0</v>
+      </c>
+      <c r="L462">
+        <v>0</v>
+      </c>
+      <c r="M462">
+        <v>30000</v>
+      </c>
+      <c r="N462">
+        <v>0</v>
+      </c>
+      <c r="O462">
+        <v>30000</v>
+      </c>
+      <c r="P462">
+        <v>4</v>
+      </c>
+      <c r="Q462">
+        <v>1.5</v>
+      </c>
+      <c r="R462" t="s">
+        <v>122</v>
+      </c>
+      <c r="S462" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="463" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A463" t="s">
+        <v>55</v>
+      </c>
+      <c r="D463" t="s">
+        <v>50</v>
+      </c>
+      <c r="H463">
+        <v>706</v>
+      </c>
+      <c r="I463" t="s">
+        <v>21</v>
+      </c>
+      <c r="J463">
+        <v>3530000</v>
+      </c>
+      <c r="K463">
+        <v>0</v>
+      </c>
+      <c r="L463">
+        <v>0</v>
+      </c>
+      <c r="M463">
+        <v>3530000</v>
+      </c>
+      <c r="N463">
+        <v>0</v>
+      </c>
+      <c r="O463">
+        <v>3530000</v>
+      </c>
+      <c r="P463">
+        <v>536</v>
+      </c>
+      <c r="Q463">
+        <v>1.32</v>
+      </c>
+      <c r="R463" t="s">
+        <v>122</v>
+      </c>
+      <c r="S463" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="464" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A464" t="s">
+        <v>57</v>
+      </c>
+      <c r="D464" t="s">
+        <v>50</v>
+      </c>
+      <c r="H464">
+        <v>104</v>
+      </c>
+      <c r="I464" t="s">
+        <v>21</v>
+      </c>
+      <c r="J464">
+        <v>728000</v>
+      </c>
+      <c r="K464">
+        <v>0</v>
+      </c>
+      <c r="L464">
+        <v>0</v>
+      </c>
+      <c r="M464">
+        <v>728000</v>
+      </c>
+      <c r="N464">
+        <v>0</v>
+      </c>
+      <c r="O464">
+        <v>728000</v>
+      </c>
+      <c r="P464">
+        <v>86</v>
+      </c>
+      <c r="Q464">
+        <v>1.21</v>
+      </c>
+      <c r="R464" t="s">
+        <v>122</v>
+      </c>
+      <c r="S464" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="465" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A465" t="s">
+        <v>58</v>
+      </c>
+      <c r="D465" t="s">
+        <v>50</v>
+      </c>
+      <c r="H465">
+        <v>37</v>
+      </c>
+      <c r="I465" t="s">
+        <v>21</v>
+      </c>
+      <c r="J465">
+        <v>185000</v>
+      </c>
+      <c r="K465">
+        <v>0</v>
+      </c>
+      <c r="L465">
+        <v>0</v>
+      </c>
+      <c r="M465">
+        <v>185000</v>
+      </c>
+      <c r="N465">
+        <v>0</v>
+      </c>
+      <c r="O465">
+        <v>185000</v>
+      </c>
+      <c r="P465">
+        <v>31</v>
+      </c>
+      <c r="Q465">
+        <v>1.19</v>
+      </c>
+      <c r="R465" t="s">
+        <v>122</v>
+      </c>
+      <c r="S465" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="466" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A466" t="s">
+        <v>60</v>
+      </c>
+      <c r="D466" t="s">
+        <v>50</v>
+      </c>
+      <c r="H466">
+        <v>121</v>
+      </c>
+      <c r="I466" t="s">
+        <v>21</v>
+      </c>
+      <c r="J466">
+        <v>605000</v>
+      </c>
+      <c r="K466">
+        <v>0</v>
+      </c>
+      <c r="L466">
+        <v>0</v>
+      </c>
+      <c r="M466">
+        <v>605000</v>
+      </c>
+      <c r="N466">
+        <v>0</v>
+      </c>
+      <c r="O466">
+        <v>605000</v>
+      </c>
+      <c r="P466">
+        <v>105</v>
+      </c>
+      <c r="Q466">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="R466" t="s">
+        <v>122</v>
+      </c>
+      <c r="S466" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="467" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A467" t="s">
+        <v>61</v>
+      </c>
+      <c r="D467" t="s">
+        <v>50</v>
+      </c>
+      <c r="H467">
+        <v>233</v>
+      </c>
+      <c r="I467" t="s">
+        <v>21</v>
+      </c>
+      <c r="J467">
+        <v>1147000</v>
+      </c>
+      <c r="K467">
+        <v>0</v>
+      </c>
+      <c r="L467">
+        <v>0</v>
+      </c>
+      <c r="M467">
+        <v>1147000</v>
+      </c>
+      <c r="N467">
+        <v>0</v>
+      </c>
+      <c r="O467">
+        <v>1147000</v>
+      </c>
+      <c r="P467">
+        <v>198</v>
+      </c>
+      <c r="Q467">
+        <v>1.18</v>
+      </c>
+      <c r="R467" t="s">
+        <v>122</v>
+      </c>
+      <c r="S467" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="468" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A468" t="s">
+        <v>62</v>
+      </c>
+      <c r="D468" t="s">
+        <v>50</v>
+      </c>
+      <c r="H468">
+        <v>429</v>
+      </c>
+      <c r="I468" t="s">
+        <v>21</v>
+      </c>
+      <c r="J468">
+        <v>2127000</v>
+      </c>
+      <c r="K468">
+        <v>0</v>
+      </c>
+      <c r="L468">
+        <v>0</v>
+      </c>
+      <c r="M468">
+        <v>2127000</v>
+      </c>
+      <c r="N468">
+        <v>0</v>
+      </c>
+      <c r="O468">
+        <v>2127000</v>
+      </c>
+      <c r="P468">
+        <v>323</v>
+      </c>
+      <c r="Q468">
+        <v>1.33</v>
+      </c>
+      <c r="R468" t="s">
+        <v>122</v>
+      </c>
+      <c r="S468" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="469" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A469" t="s">
+        <v>63</v>
+      </c>
+      <c r="D469" t="s">
+        <v>50</v>
+      </c>
+      <c r="H469">
+        <v>134</v>
+      </c>
+      <c r="I469" t="s">
+        <v>21</v>
+      </c>
+      <c r="J469">
+        <v>670000</v>
+      </c>
+      <c r="K469">
+        <v>0</v>
+      </c>
+      <c r="L469">
+        <v>0</v>
+      </c>
+      <c r="M469">
+        <v>670000</v>
+      </c>
+      <c r="N469">
+        <v>0</v>
+      </c>
+      <c r="O469">
+        <v>670000</v>
+      </c>
+      <c r="P469">
+        <v>115</v>
+      </c>
+      <c r="Q469">
+        <v>1.17</v>
+      </c>
+      <c r="R469" t="s">
+        <v>122</v>
+      </c>
+      <c r="S469" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="470" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A470" t="s">
+        <v>79</v>
+      </c>
+      <c r="D470" t="s">
+        <v>50</v>
+      </c>
+      <c r="H470">
+        <v>56</v>
+      </c>
+      <c r="I470" t="s">
+        <v>21</v>
+      </c>
+      <c r="J470">
+        <v>168000</v>
+      </c>
+      <c r="K470">
+        <v>0</v>
+      </c>
+      <c r="L470">
+        <v>0</v>
+      </c>
+      <c r="M470">
+        <v>168000</v>
+      </c>
+      <c r="N470">
+        <v>0</v>
+      </c>
+      <c r="O470">
+        <v>168000</v>
+      </c>
+      <c r="P470">
+        <v>20</v>
+      </c>
+      <c r="Q470">
+        <v>2.8</v>
+      </c>
+      <c r="R470" t="s">
+        <v>122</v>
+      </c>
+      <c r="S470" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="471" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A471" t="s">
+        <v>65</v>
+      </c>
+      <c r="D471" t="s">
+        <v>50</v>
+      </c>
+      <c r="H471">
+        <v>112</v>
+      </c>
+      <c r="I471" t="s">
+        <v>21</v>
+      </c>
+      <c r="J471">
+        <v>448000</v>
+      </c>
+      <c r="K471">
+        <v>0</v>
+      </c>
+      <c r="L471">
+        <v>0</v>
+      </c>
+      <c r="M471">
+        <v>448000</v>
+      </c>
+      <c r="N471">
+        <v>0</v>
+      </c>
+      <c r="O471">
+        <v>448000</v>
+      </c>
+      <c r="P471">
+        <v>52</v>
+      </c>
+      <c r="Q471">
+        <v>2.15</v>
+      </c>
+      <c r="R471" t="s">
+        <v>122</v>
+      </c>
+      <c r="S471" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="472" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A472" t="s">
+        <v>66</v>
+      </c>
+      <c r="D472" t="s">
+        <v>50</v>
+      </c>
+      <c r="H472">
+        <v>74</v>
+      </c>
+      <c r="I472" t="s">
+        <v>21</v>
+      </c>
+      <c r="J472">
+        <v>1332000</v>
+      </c>
+      <c r="K472">
+        <v>0</v>
+      </c>
+      <c r="L472">
+        <v>0</v>
+      </c>
+      <c r="M472">
+        <v>1332000</v>
+      </c>
+      <c r="N472">
+        <v>0</v>
+      </c>
+      <c r="O472">
+        <v>1332000</v>
+      </c>
+      <c r="P472">
+        <v>66</v>
+      </c>
+      <c r="Q472">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="R472" t="s">
+        <v>122</v>
+      </c>
+      <c r="S472" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="473" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A473" t="s">
+        <v>80</v>
+      </c>
+      <c r="D473" t="s">
+        <v>50</v>
+      </c>
+      <c r="H473">
+        <v>49</v>
+      </c>
+      <c r="I473" t="s">
+        <v>21</v>
+      </c>
+      <c r="J473">
+        <v>245000</v>
+      </c>
+      <c r="K473">
+        <v>0</v>
+      </c>
+      <c r="L473">
+        <v>0</v>
+      </c>
+      <c r="M473">
+        <v>245000</v>
+      </c>
+      <c r="N473">
+        <v>0</v>
+      </c>
+      <c r="O473">
+        <v>245000</v>
+      </c>
+      <c r="P473">
+        <v>23</v>
+      </c>
+      <c r="Q473">
+        <v>2.13</v>
+      </c>
+      <c r="R473" t="s">
+        <v>122</v>
+      </c>
+      <c r="S473" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="474" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A474" t="s">
+        <v>81</v>
+      </c>
+      <c r="D474" t="s">
+        <v>50</v>
+      </c>
+      <c r="H474">
+        <v>66</v>
+      </c>
+      <c r="I474" t="s">
+        <v>21</v>
+      </c>
+      <c r="J474">
+        <v>330000</v>
+      </c>
+      <c r="K474">
+        <v>0</v>
+      </c>
+      <c r="L474">
+        <v>0</v>
+      </c>
+      <c r="M474">
+        <v>330000</v>
+      </c>
+      <c r="N474">
+        <v>0</v>
+      </c>
+      <c r="O474">
+        <v>330000</v>
+      </c>
+      <c r="P474">
+        <v>42</v>
+      </c>
+      <c r="Q474">
+        <v>1.57</v>
+      </c>
+      <c r="R474" t="s">
+        <v>122</v>
+      </c>
+      <c r="S474" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="475" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A475" t="s">
+        <v>67</v>
+      </c>
+      <c r="D475" t="s">
+        <v>50</v>
+      </c>
+      <c r="H475">
+        <v>223</v>
+      </c>
+      <c r="I475" t="s">
+        <v>21</v>
+      </c>
+      <c r="J475">
+        <v>883000</v>
+      </c>
+      <c r="K475">
+        <v>0</v>
+      </c>
+      <c r="L475">
+        <v>0</v>
+      </c>
+      <c r="M475">
+        <v>883000</v>
+      </c>
+      <c r="N475">
+        <v>0</v>
+      </c>
+      <c r="O475">
+        <v>883000</v>
+      </c>
+      <c r="P475">
+        <v>180</v>
+      </c>
+      <c r="Q475">
+        <v>1.24</v>
+      </c>
+      <c r="R475" t="s">
+        <v>122</v>
+      </c>
+      <c r="S475" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="476" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A476" t="s">
+        <v>68</v>
+      </c>
+      <c r="D476" t="s">
+        <v>50</v>
+      </c>
+      <c r="H476">
+        <v>33</v>
+      </c>
+      <c r="I476" t="s">
+        <v>21</v>
+      </c>
+      <c r="J476">
+        <v>163000</v>
+      </c>
+      <c r="K476">
+        <v>0</v>
+      </c>
+      <c r="L476">
+        <v>0</v>
+      </c>
+      <c r="M476">
+        <v>163000</v>
+      </c>
+      <c r="N476">
+        <v>0</v>
+      </c>
+      <c r="O476">
+        <v>163000</v>
+      </c>
+      <c r="P476">
+        <v>26</v>
+      </c>
+      <c r="Q476">
+        <v>1.27</v>
+      </c>
+      <c r="R476" t="s">
+        <v>122</v>
+      </c>
+      <c r="S476" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="477" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A477" t="s">
+        <v>69</v>
+      </c>
+      <c r="D477" t="s">
+        <v>50</v>
+      </c>
+      <c r="H477">
+        <v>96</v>
+      </c>
+      <c r="I477" t="s">
+        <v>21</v>
+      </c>
+      <c r="J477">
+        <v>480000</v>
+      </c>
+      <c r="K477">
+        <v>0</v>
+      </c>
+      <c r="L477">
+        <v>0</v>
+      </c>
+      <c r="M477">
+        <v>480000</v>
+      </c>
+      <c r="N477">
+        <v>0</v>
+      </c>
+      <c r="O477">
+        <v>480000</v>
+      </c>
+      <c r="P477">
+        <v>80</v>
+      </c>
+      <c r="Q477">
+        <v>1.2</v>
+      </c>
+      <c r="R477" t="s">
+        <v>122</v>
+      </c>
+      <c r="S477" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="478" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A478" t="s">
+        <v>70</v>
+      </c>
+      <c r="D478" t="s">
+        <v>71</v>
+      </c>
+      <c r="H478">
+        <v>136</v>
+      </c>
+      <c r="I478" t="s">
+        <v>21</v>
+      </c>
+      <c r="J478">
+        <v>1632000</v>
+      </c>
+      <c r="K478">
+        <v>0</v>
+      </c>
+      <c r="L478">
+        <v>0</v>
+      </c>
+      <c r="M478">
+        <v>1632000</v>
+      </c>
+      <c r="N478">
+        <v>0</v>
+      </c>
+      <c r="O478">
+        <v>1632000</v>
+      </c>
+      <c r="P478">
+        <v>132</v>
+      </c>
+      <c r="Q478">
+        <v>1.03</v>
+      </c>
+      <c r="R478" t="s">
+        <v>122</v>
+      </c>
+      <c r="S478" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="479" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A479" t="s">
+        <v>72</v>
+      </c>
+      <c r="D479" t="s">
+        <v>71</v>
+      </c>
+      <c r="H479">
+        <v>184</v>
+      </c>
+      <c r="I479" t="s">
+        <v>21</v>
+      </c>
+      <c r="J479">
+        <v>2208000</v>
+      </c>
+      <c r="K479">
+        <v>0</v>
+      </c>
+      <c r="L479">
+        <v>0</v>
+      </c>
+      <c r="M479">
+        <v>2208000</v>
+      </c>
+      <c r="N479">
+        <v>0</v>
+      </c>
+      <c r="O479">
+        <v>2208000</v>
+      </c>
+      <c r="P479">
+        <v>177</v>
+      </c>
+      <c r="Q479">
+        <v>1.04</v>
+      </c>
+      <c r="R479" t="s">
+        <v>122</v>
+      </c>
+      <c r="S479" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="480" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A480" t="s">
+        <v>82</v>
+      </c>
+      <c r="D480" t="s">
+        <v>71</v>
+      </c>
+      <c r="H480">
+        <v>11</v>
+      </c>
+      <c r="I480" t="s">
+        <v>21</v>
+      </c>
+      <c r="J480">
+        <v>66000</v>
+      </c>
+      <c r="K480">
+        <v>0</v>
+      </c>
+      <c r="L480">
+        <v>0</v>
+      </c>
+      <c r="M480">
+        <v>66000</v>
+      </c>
+      <c r="N480">
+        <v>0</v>
+      </c>
+      <c r="O480">
+        <v>66000</v>
+      </c>
+      <c r="P480">
+        <v>11</v>
+      </c>
+      <c r="Q480">
+        <v>1</v>
+      </c>
+      <c r="R480" t="s">
+        <v>122</v>
+      </c>
+      <c r="S480" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="481" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A481" t="s">
+        <v>73</v>
+      </c>
+      <c r="D481" t="s">
+        <v>71</v>
+      </c>
+      <c r="H481">
+        <v>102</v>
+      </c>
+      <c r="I481" t="s">
+        <v>21</v>
+      </c>
+      <c r="J481">
+        <v>1216000</v>
+      </c>
+      <c r="K481">
+        <v>0</v>
+      </c>
+      <c r="L481">
+        <v>0</v>
+      </c>
+      <c r="M481">
+        <v>1216000</v>
+      </c>
+      <c r="N481">
+        <v>0</v>
+      </c>
+      <c r="O481">
+        <v>1216000</v>
+      </c>
+      <c r="P481">
+        <v>100</v>
+      </c>
+      <c r="Q481">
+        <v>1.02</v>
+      </c>
+      <c r="R481" t="s">
+        <v>122</v>
+      </c>
+      <c r="S481" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="482" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A482" t="s">
+        <v>83</v>
+      </c>
+      <c r="D482" t="s">
+        <v>71</v>
+      </c>
+      <c r="H482">
+        <v>2</v>
+      </c>
+      <c r="I482" t="s">
+        <v>21</v>
+      </c>
+      <c r="J482">
+        <v>12000</v>
+      </c>
+      <c r="K482">
+        <v>0</v>
+      </c>
+      <c r="L482">
+        <v>0</v>
+      </c>
+      <c r="M482">
+        <v>12000</v>
+      </c>
+      <c r="N482">
+        <v>0</v>
+      </c>
+      <c r="O482">
+        <v>12000</v>
+      </c>
+      <c r="P482">
+        <v>2</v>
+      </c>
+      <c r="Q482">
+        <v>1</v>
+      </c>
+      <c r="R482" t="s">
+        <v>122</v>
+      </c>
+      <c r="S482" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="483" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A483" t="s">
+        <v>75</v>
+      </c>
+      <c r="D483" t="s">
+        <v>71</v>
+      </c>
+      <c r="H483">
+        <v>135</v>
+      </c>
+      <c r="I483" t="s">
+        <v>21</v>
+      </c>
+      <c r="J483">
+        <v>1620000</v>
+      </c>
+      <c r="K483">
+        <v>0</v>
+      </c>
+      <c r="L483">
+        <v>0</v>
+      </c>
+      <c r="M483">
+        <v>1620000</v>
+      </c>
+      <c r="N483">
+        <v>0</v>
+      </c>
+      <c r="O483">
+        <v>1620000</v>
+      </c>
+      <c r="P483">
+        <v>130</v>
+      </c>
+      <c r="Q483">
+        <v>1.04</v>
+      </c>
+      <c r="R483" t="s">
+        <v>122</v>
+      </c>
+      <c r="S483" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="484" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A484" t="s">
+        <v>76</v>
+      </c>
+      <c r="D484" t="s">
+        <v>71</v>
+      </c>
+      <c r="H484">
+        <v>58</v>
+      </c>
+      <c r="I484" t="s">
+        <v>21</v>
+      </c>
+      <c r="J484">
+        <v>696000</v>
+      </c>
+      <c r="K484">
+        <v>0</v>
+      </c>
+      <c r="L484">
+        <v>0</v>
+      </c>
+      <c r="M484">
+        <v>696000</v>
+      </c>
+      <c r="N484">
+        <v>0</v>
+      </c>
+      <c r="O484">
+        <v>696000</v>
+      </c>
+      <c r="P484">
+        <v>57</v>
+      </c>
+      <c r="Q484">
+        <v>1.02</v>
+      </c>
+      <c r="R484" t="s">
+        <v>122</v>
+      </c>
+      <c r="S484" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="485" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A485" t="s">
+        <v>77</v>
+      </c>
+      <c r="D485" t="s">
+        <v>71</v>
+      </c>
+      <c r="H485">
+        <v>58</v>
+      </c>
+      <c r="I485" t="s">
+        <v>21</v>
+      </c>
+      <c r="J485">
+        <v>696000</v>
+      </c>
+      <c r="K485">
+        <v>0</v>
+      </c>
+      <c r="L485">
+        <v>0</v>
+      </c>
+      <c r="M485">
+        <v>696000</v>
+      </c>
+      <c r="N485">
+        <v>0</v>
+      </c>
+      <c r="O485">
+        <v>696000</v>
+      </c>
+      <c r="P485">
+        <v>58</v>
+      </c>
+      <c r="Q485">
+        <v>1</v>
+      </c>
+      <c r="R485" t="s">
+        <v>122</v>
+      </c>
+      <c r="S485" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="486" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A486" t="s">
+        <v>84</v>
+      </c>
+      <c r="D486" t="s">
+        <v>71</v>
+      </c>
+      <c r="H486">
+        <v>7</v>
+      </c>
+      <c r="I486" t="s">
+        <v>21</v>
+      </c>
+      <c r="J486">
+        <v>42000</v>
+      </c>
+      <c r="K486">
+        <v>0</v>
+      </c>
+      <c r="L486">
+        <v>0</v>
+      </c>
+      <c r="M486">
+        <v>42000</v>
+      </c>
+      <c r="N486">
+        <v>0</v>
+      </c>
+      <c r="O486">
+        <v>42000</v>
+      </c>
+      <c r="P486">
+        <v>7</v>
+      </c>
+      <c r="Q486">
+        <v>1</v>
+      </c>
+      <c r="R486" t="s">
+        <v>122</v>
+      </c>
+      <c r="S486" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="487" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A487" t="s">
+        <v>19</v>
+      </c>
+      <c r="D487" t="s">
+        <v>20</v>
+      </c>
+      <c r="H487">
+        <v>207</v>
+      </c>
+      <c r="I487" t="s">
+        <v>21</v>
+      </c>
+      <c r="J487">
+        <v>4035000</v>
+      </c>
+      <c r="K487">
+        <v>0</v>
+      </c>
+      <c r="L487">
+        <v>0</v>
+      </c>
+      <c r="M487">
+        <v>4035000</v>
+      </c>
+      <c r="N487">
+        <v>0</v>
+      </c>
+      <c r="O487">
+        <v>4035000</v>
+      </c>
+      <c r="P487">
+        <v>163</v>
+      </c>
+      <c r="Q487">
+        <v>1.27</v>
+      </c>
+      <c r="R487" t="s">
+        <v>122</v>
+      </c>
+      <c r="S487" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="488" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A488" t="s">
+        <v>89</v>
+      </c>
+      <c r="D488" t="s">
+        <v>25</v>
+      </c>
+      <c r="H488">
+        <v>86</v>
+      </c>
+      <c r="I488" t="s">
+        <v>21</v>
+      </c>
+      <c r="J488">
+        <v>2752000</v>
+      </c>
+      <c r="K488">
+        <v>0</v>
+      </c>
+      <c r="L488">
+        <v>0</v>
+      </c>
+      <c r="M488">
+        <v>2752000</v>
+      </c>
+      <c r="N488">
+        <v>1633293.94</v>
+      </c>
+      <c r="O488">
+        <v>1118706.06</v>
+      </c>
+      <c r="P488">
+        <v>64</v>
+      </c>
+      <c r="Q488">
+        <v>1.34</v>
+      </c>
+      <c r="R488" t="s">
+        <v>122</v>
+      </c>
+      <c r="S488" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="489" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A489" t="s">
+        <v>27</v>
+      </c>
+      <c r="D489" t="s">
+        <v>25</v>
+      </c>
+      <c r="H489">
+        <v>170</v>
+      </c>
+      <c r="I489" t="s">
+        <v>21</v>
+      </c>
+      <c r="J489">
+        <v>4250000</v>
+      </c>
+      <c r="K489">
+        <v>0</v>
+      </c>
+      <c r="L489">
+        <v>0</v>
+      </c>
+      <c r="M489">
+        <v>4250000</v>
+      </c>
+      <c r="N489">
+        <v>1409604.3</v>
+      </c>
+      <c r="O489">
+        <v>2840395.7</v>
+      </c>
+      <c r="P489">
+        <v>123</v>
+      </c>
+      <c r="Q489">
+        <v>1.38</v>
+      </c>
+      <c r="R489" t="s">
+        <v>122</v>
+      </c>
+      <c r="S489" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="490" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A490" t="s">
+        <v>28</v>
+      </c>
+      <c r="D490" t="s">
+        <v>25</v>
+      </c>
+      <c r="H490">
+        <v>143</v>
+      </c>
+      <c r="I490" t="s">
+        <v>21</v>
+      </c>
+      <c r="J490">
+        <v>2564000</v>
+      </c>
+      <c r="K490">
+        <v>0</v>
+      </c>
+      <c r="L490">
+        <v>0</v>
+      </c>
+      <c r="M490">
+        <v>2564000</v>
+      </c>
+      <c r="N490">
+        <v>96149165.969999999</v>
+      </c>
+      <c r="O490">
+        <v>-93585165.969999999</v>
+      </c>
+      <c r="P490">
+        <v>119</v>
+      </c>
+      <c r="Q490">
+        <v>1.2</v>
+      </c>
+      <c r="R490" t="s">
+        <v>122</v>
+      </c>
+      <c r="S490" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="491" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A491" t="s">
+        <v>90</v>
+      </c>
+      <c r="D491" t="s">
+        <v>25</v>
+      </c>
+      <c r="H491">
+        <v>1</v>
+      </c>
+      <c r="I491" t="s">
+        <v>21</v>
+      </c>
+      <c r="J491">
+        <v>20000</v>
+      </c>
+      <c r="K491">
+        <v>0</v>
+      </c>
+      <c r="L491">
+        <v>0</v>
+      </c>
+      <c r="M491">
+        <v>20000</v>
+      </c>
+      <c r="N491">
+        <v>26891.79</v>
+      </c>
+      <c r="O491">
+        <v>-6891.79</v>
+      </c>
+      <c r="P491">
+        <v>1</v>
+      </c>
+      <c r="Q491">
+        <v>1</v>
+      </c>
+      <c r="R491" t="s">
+        <v>122</v>
+      </c>
+      <c r="S491" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="492" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A492" t="s">
+        <v>30</v>
+      </c>
+      <c r="D492" t="s">
+        <v>25</v>
+      </c>
+      <c r="H492">
+        <v>83</v>
+      </c>
+      <c r="I492" t="s">
+        <v>21</v>
+      </c>
+      <c r="J492">
+        <v>1660000</v>
+      </c>
+      <c r="K492">
+        <v>0</v>
+      </c>
+      <c r="L492">
+        <v>0</v>
+      </c>
+      <c r="M492">
+        <v>1660000</v>
+      </c>
+      <c r="N492">
+        <v>55931358.57</v>
+      </c>
+      <c r="O492">
+        <v>-54271358.57</v>
+      </c>
+      <c r="P492">
+        <v>75</v>
+      </c>
+      <c r="Q492">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="R492" t="s">
+        <v>122</v>
+      </c>
+      <c r="S492" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="493" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A493" t="s">
+        <v>31</v>
+      </c>
+      <c r="D493" t="s">
+        <v>25</v>
+      </c>
+      <c r="H493">
+        <v>274</v>
+      </c>
+      <c r="I493" t="s">
+        <v>21</v>
+      </c>
+      <c r="J493">
+        <v>8217000</v>
+      </c>
+      <c r="K493">
+        <v>0</v>
+      </c>
+      <c r="L493">
+        <v>0</v>
+      </c>
+      <c r="M493">
+        <v>8217000</v>
+      </c>
+      <c r="N493">
+        <v>2189750.46</v>
+      </c>
+      <c r="O493">
+        <v>6027249.54</v>
+      </c>
+      <c r="P493">
+        <v>207</v>
+      </c>
+      <c r="Q493">
+        <v>1.32</v>
+      </c>
+      <c r="R493" t="s">
+        <v>122</v>
+      </c>
+      <c r="S493" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="494" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A494" t="s">
+        <v>33</v>
+      </c>
+      <c r="D494" t="s">
+        <v>25</v>
+      </c>
+      <c r="H494">
+        <v>104</v>
+      </c>
+      <c r="I494" t="s">
+        <v>21</v>
+      </c>
+      <c r="J494">
+        <v>2392000</v>
+      </c>
+      <c r="K494">
+        <v>0</v>
+      </c>
+      <c r="L494">
+        <v>0</v>
+      </c>
+      <c r="M494">
+        <v>2392000</v>
+      </c>
+      <c r="N494">
+        <v>69614666.159999996</v>
+      </c>
+      <c r="O494">
+        <v>-67222666.159999996</v>
+      </c>
+      <c r="P494">
+        <v>88</v>
+      </c>
+      <c r="Q494">
+        <v>1.18</v>
+      </c>
+      <c r="R494" t="s">
+        <v>122</v>
+      </c>
+      <c r="S494" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="495" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A495" t="s">
+        <v>35</v>
+      </c>
+      <c r="D495" t="s">
+        <v>25</v>
+      </c>
+      <c r="H495">
+        <v>167</v>
+      </c>
+      <c r="I495" t="s">
+        <v>21</v>
+      </c>
+      <c r="J495">
+        <v>3336000</v>
+      </c>
+      <c r="K495">
+        <v>0</v>
+      </c>
+      <c r="L495">
+        <v>0</v>
+      </c>
+      <c r="M495">
+        <v>3336000</v>
+      </c>
+      <c r="N495">
+        <v>365694.93</v>
+      </c>
+      <c r="O495">
+        <v>2970305.07</v>
+      </c>
+      <c r="P495">
+        <v>130</v>
+      </c>
+      <c r="Q495">
+        <v>1.28</v>
+      </c>
+      <c r="R495" t="s">
+        <v>122</v>
+      </c>
+      <c r="S495" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="496" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A496" t="s">
+        <v>36</v>
+      </c>
+      <c r="D496" t="s">
+        <v>25</v>
+      </c>
+      <c r="H496">
+        <v>195</v>
+      </c>
+      <c r="I496" t="s">
+        <v>21</v>
+      </c>
+      <c r="J496">
+        <v>4875000</v>
+      </c>
+      <c r="K496">
+        <v>0</v>
+      </c>
+      <c r="L496">
+        <v>0</v>
+      </c>
+      <c r="M496">
+        <v>4875000</v>
+      </c>
+      <c r="N496">
+        <v>895009.05</v>
+      </c>
+      <c r="O496">
+        <v>3979990.95</v>
+      </c>
+      <c r="P496">
+        <v>155</v>
+      </c>
+      <c r="Q496">
+        <v>1.26</v>
+      </c>
+      <c r="R496" t="s">
+        <v>122</v>
+      </c>
+      <c r="S496" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="497" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A497" t="s">
+        <v>110</v>
+      </c>
+      <c r="D497" t="s">
+        <v>44</v>
+      </c>
+      <c r="H497">
+        <v>318</v>
+      </c>
+      <c r="I497" t="s">
+        <v>21</v>
+      </c>
+      <c r="J497">
+        <v>1590000</v>
+      </c>
+      <c r="K497">
+        <v>0</v>
+      </c>
+      <c r="L497">
+        <v>0</v>
+      </c>
+      <c r="M497">
+        <v>1590000</v>
+      </c>
+      <c r="N497">
+        <v>528986.64</v>
+      </c>
+      <c r="O497">
+        <v>1061013.3600000001</v>
+      </c>
+      <c r="P497">
+        <v>248</v>
+      </c>
+      <c r="Q497">
+        <v>1.28</v>
+      </c>
+      <c r="R497" t="s">
+        <v>122</v>
+      </c>
+      <c r="S497" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="498" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A498" t="s">
+        <v>46</v>
+      </c>
+      <c r="D498" t="s">
+        <v>44</v>
+      </c>
+      <c r="H498">
+        <v>8</v>
+      </c>
+      <c r="I498" t="s">
+        <v>21</v>
+      </c>
+      <c r="J498">
+        <v>120000</v>
+      </c>
+      <c r="K498">
+        <v>0</v>
+      </c>
+      <c r="L498">
+        <v>0</v>
+      </c>
+      <c r="M498">
+        <v>120000</v>
+      </c>
+      <c r="N498">
+        <v>0</v>
+      </c>
+      <c r="O498">
+        <v>120000</v>
+      </c>
+      <c r="P498">
+        <v>6</v>
+      </c>
+      <c r="Q498">
+        <v>1.33</v>
+      </c>
+      <c r="R498" t="s">
+        <v>122</v>
+      </c>
+      <c r="S498" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="499" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A499" t="s">
+        <v>111</v>
+      </c>
+      <c r="D499" t="s">
+        <v>44</v>
+      </c>
+      <c r="H499">
+        <v>149</v>
+      </c>
+      <c r="I499" t="s">
+        <v>21</v>
+      </c>
+      <c r="J499">
+        <v>745000</v>
+      </c>
+      <c r="K499">
+        <v>0</v>
+      </c>
+      <c r="L499">
+        <v>0</v>
+      </c>
+      <c r="M499">
+        <v>745000</v>
+      </c>
+      <c r="N499">
+        <v>322883</v>
+      </c>
+      <c r="O499">
+        <v>422117</v>
+      </c>
+      <c r="P499">
+        <v>91</v>
+      </c>
+      <c r="Q499">
+        <v>1.64</v>
+      </c>
+      <c r="R499" t="s">
+        <v>122</v>
+      </c>
+      <c r="S499" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="500" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A500" t="s">
+        <v>55</v>
+      </c>
+      <c r="D500" t="s">
+        <v>50</v>
+      </c>
+      <c r="H500">
+        <v>264</v>
+      </c>
+      <c r="I500" t="s">
+        <v>21</v>
+      </c>
+      <c r="J500">
+        <v>1320000</v>
+      </c>
+      <c r="K500">
+        <v>0</v>
+      </c>
+      <c r="L500">
+        <v>0</v>
+      </c>
+      <c r="M500">
+        <v>1320000</v>
+      </c>
+      <c r="N500">
+        <v>528000</v>
+      </c>
+      <c r="O500">
+        <v>792000</v>
+      </c>
+      <c r="P500">
+        <v>182</v>
+      </c>
+      <c r="Q500">
+        <v>1.45</v>
+      </c>
+      <c r="R500" t="s">
+        <v>122</v>
+      </c>
+      <c r="S500" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="501" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A501" t="s">
+        <v>119</v>
+      </c>
+      <c r="D501" t="s">
+        <v>50</v>
+      </c>
+      <c r="H501">
+        <v>61</v>
+      </c>
+      <c r="I501" t="s">
+        <v>21</v>
+      </c>
+      <c r="J501">
+        <v>427000</v>
+      </c>
+      <c r="K501">
+        <v>0</v>
+      </c>
+      <c r="L501">
+        <v>0</v>
+      </c>
+      <c r="M501">
+        <v>427000</v>
+      </c>
+      <c r="N501">
+        <v>0</v>
+      </c>
+      <c r="O501">
+        <v>427000</v>
+      </c>
+      <c r="P501">
+        <v>50</v>
+      </c>
+      <c r="Q501">
+        <v>1.22</v>
+      </c>
+      <c r="R501" t="s">
+        <v>122</v>
+      </c>
+      <c r="S501" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="502" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A502" t="s">
+        <v>58</v>
+      </c>
+      <c r="D502" t="s">
+        <v>50</v>
+      </c>
+      <c r="H502">
+        <v>38</v>
+      </c>
+      <c r="I502" t="s">
+        <v>21</v>
+      </c>
+      <c r="J502">
+        <v>190000</v>
+      </c>
+      <c r="K502">
+        <v>0</v>
+      </c>
+      <c r="L502">
+        <v>0</v>
+      </c>
+      <c r="M502">
+        <v>190000</v>
+      </c>
+      <c r="N502">
+        <v>152000</v>
+      </c>
+      <c r="O502">
+        <v>38000</v>
+      </c>
+      <c r="P502">
+        <v>30</v>
+      </c>
+      <c r="Q502">
+        <v>1.27</v>
+      </c>
+      <c r="R502" t="s">
+        <v>122</v>
+      </c>
+      <c r="S502" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="503" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A503" t="s">
+        <v>61</v>
+      </c>
+      <c r="D503" t="s">
+        <v>50</v>
+      </c>
+      <c r="H503">
+        <v>126</v>
+      </c>
+      <c r="I503" t="s">
+        <v>21</v>
+      </c>
+      <c r="J503">
+        <v>626000</v>
+      </c>
+      <c r="K503">
+        <v>0</v>
+      </c>
+      <c r="L503">
+        <v>0</v>
+      </c>
+      <c r="M503">
+        <v>626000</v>
+      </c>
+      <c r="N503">
+        <v>0</v>
+      </c>
+      <c r="O503">
+        <v>626000</v>
+      </c>
+      <c r="P503">
+        <v>105</v>
+      </c>
+      <c r="Q503">
+        <v>1.2</v>
+      </c>
+      <c r="R503" t="s">
+        <v>122</v>
+      </c>
+      <c r="S503" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="504" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A504" t="s">
+        <v>62</v>
+      </c>
+      <c r="D504" t="s">
+        <v>50</v>
+      </c>
+      <c r="H504">
+        <v>216</v>
+      </c>
+      <c r="I504" t="s">
+        <v>21</v>
+      </c>
+      <c r="J504">
+        <v>1078000</v>
+      </c>
+      <c r="K504">
+        <v>0</v>
+      </c>
+      <c r="L504">
+        <v>0</v>
+      </c>
+      <c r="M504">
+        <v>1078000</v>
+      </c>
+      <c r="N504">
+        <v>0</v>
+      </c>
+      <c r="O504">
+        <v>1078000</v>
+      </c>
+      <c r="P504">
+        <v>160</v>
+      </c>
+      <c r="Q504">
+        <v>1.35</v>
+      </c>
+      <c r="R504" t="s">
+        <v>122</v>
+      </c>
+      <c r="S504" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="505" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A505" t="s">
+        <v>63</v>
+      </c>
+      <c r="D505" t="s">
+        <v>50</v>
+      </c>
+      <c r="H505">
+        <v>60</v>
+      </c>
+      <c r="I505" t="s">
+        <v>21</v>
+      </c>
+      <c r="J505">
+        <v>300000</v>
+      </c>
+      <c r="K505">
+        <v>0</v>
+      </c>
+      <c r="L505">
+        <v>0</v>
+      </c>
+      <c r="M505">
+        <v>300000</v>
+      </c>
+      <c r="N505">
+        <v>0</v>
+      </c>
+      <c r="O505">
+        <v>300000</v>
+      </c>
+      <c r="P505">
+        <v>54</v>
+      </c>
+      <c r="Q505">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="R505" t="s">
+        <v>122</v>
+      </c>
+      <c r="S505" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="506" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A506" t="s">
+        <v>64</v>
+      </c>
+      <c r="D506" t="s">
+        <v>50</v>
+      </c>
+      <c r="H506">
+        <v>6</v>
+      </c>
+      <c r="I506" t="s">
+        <v>21</v>
+      </c>
+      <c r="J506">
+        <v>108000</v>
+      </c>
+      <c r="K506">
+        <v>0</v>
+      </c>
+      <c r="L506">
+        <v>0</v>
+      </c>
+      <c r="M506">
+        <v>108000</v>
+      </c>
+      <c r="N506">
+        <v>0</v>
+      </c>
+      <c r="O506">
+        <v>108000</v>
+      </c>
+      <c r="P506">
+        <v>6</v>
+      </c>
+      <c r="Q506">
+        <v>1</v>
+      </c>
+      <c r="R506" t="s">
+        <v>122</v>
+      </c>
+      <c r="S506" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="507" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A507" t="s">
+        <v>79</v>
+      </c>
+      <c r="D507" t="s">
+        <v>50</v>
+      </c>
+      <c r="H507">
+        <v>109</v>
+      </c>
+      <c r="I507" t="s">
+        <v>21</v>
+      </c>
+      <c r="J507">
+        <v>327000</v>
+      </c>
+      <c r="K507">
+        <v>0</v>
+      </c>
+      <c r="L507">
+        <v>0</v>
+      </c>
+      <c r="M507">
+        <v>327000</v>
+      </c>
+      <c r="N507">
+        <v>0</v>
+      </c>
+      <c r="O507">
+        <v>327000</v>
+      </c>
+      <c r="P507">
+        <v>33</v>
+      </c>
+      <c r="Q507">
+        <v>3.3</v>
+      </c>
+      <c r="R507" t="s">
+        <v>122</v>
+      </c>
+      <c r="S507" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="508" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A508" t="s">
+        <v>65</v>
+      </c>
+      <c r="D508" t="s">
+        <v>50</v>
+      </c>
+      <c r="H508">
+        <v>35</v>
+      </c>
+      <c r="I508" t="s">
+        <v>21</v>
+      </c>
+      <c r="J508">
+        <v>140000</v>
+      </c>
+      <c r="K508">
+        <v>0</v>
+      </c>
+      <c r="L508">
+        <v>0</v>
+      </c>
+      <c r="M508">
+        <v>140000</v>
+      </c>
+      <c r="N508">
+        <v>0</v>
+      </c>
+      <c r="O508">
+        <v>140000</v>
+      </c>
+      <c r="P508">
+        <v>20</v>
+      </c>
+      <c r="Q508">
+        <v>1.75</v>
+      </c>
+      <c r="R508" t="s">
+        <v>122</v>
+      </c>
+      <c r="S508" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="509" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A509" t="s">
+        <v>66</v>
+      </c>
+      <c r="D509" t="s">
+        <v>50</v>
+      </c>
+      <c r="H509">
+        <v>21</v>
+      </c>
+      <c r="I509" t="s">
+        <v>21</v>
+      </c>
+      <c r="J509">
+        <v>378000</v>
+      </c>
+      <c r="K509">
+        <v>0</v>
+      </c>
+      <c r="L509">
+        <v>0</v>
+      </c>
+      <c r="M509">
+        <v>378000</v>
+      </c>
+      <c r="N509">
+        <v>0</v>
+      </c>
+      <c r="O509">
+        <v>378000</v>
+      </c>
+      <c r="P509">
+        <v>19</v>
+      </c>
+      <c r="Q509">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="R509" t="s">
+        <v>122</v>
+      </c>
+      <c r="S509" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="510" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A510" t="s">
+        <v>80</v>
+      </c>
+      <c r="D510" t="s">
+        <v>50</v>
+      </c>
+      <c r="H510">
+        <v>68</v>
+      </c>
+      <c r="I510" t="s">
+        <v>21</v>
+      </c>
+      <c r="J510">
+        <v>340000</v>
+      </c>
+      <c r="K510">
+        <v>0</v>
+      </c>
+      <c r="L510">
+        <v>0</v>
+      </c>
+      <c r="M510">
+        <v>340000</v>
+      </c>
+      <c r="N510">
+        <v>0</v>
+      </c>
+      <c r="O510">
+        <v>340000</v>
+      </c>
+      <c r="P510">
+        <v>45</v>
+      </c>
+      <c r="Q510">
+        <v>1.51</v>
+      </c>
+      <c r="R510" t="s">
+        <v>122</v>
+      </c>
+      <c r="S510" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="511" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A511" t="s">
+        <v>81</v>
+      </c>
+      <c r="D511" t="s">
+        <v>50</v>
+      </c>
+      <c r="H511">
+        <v>24</v>
+      </c>
+      <c r="I511" t="s">
+        <v>21</v>
+      </c>
+      <c r="J511">
+        <v>120000</v>
+      </c>
+      <c r="K511">
+        <v>0</v>
+      </c>
+      <c r="L511">
+        <v>0</v>
+      </c>
+      <c r="M511">
+        <v>120000</v>
+      </c>
+      <c r="N511">
+        <v>0</v>
+      </c>
+      <c r="O511">
+        <v>120000</v>
+      </c>
+      <c r="P511">
+        <v>10</v>
+      </c>
+      <c r="Q511">
+        <v>2.4</v>
+      </c>
+      <c r="R511" t="s">
+        <v>122</v>
+      </c>
+      <c r="S511" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="512" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A512" t="s">
+        <v>112</v>
+      </c>
+      <c r="D512" t="s">
+        <v>50</v>
+      </c>
+      <c r="H512">
+        <v>7</v>
+      </c>
+      <c r="I512" t="s">
+        <v>21</v>
+      </c>
+      <c r="J512">
+        <v>28000</v>
+      </c>
+      <c r="K512">
+        <v>0</v>
+      </c>
+      <c r="L512">
+        <v>0</v>
+      </c>
+      <c r="M512">
+        <v>28000</v>
+      </c>
+      <c r="N512">
+        <v>116.9</v>
+      </c>
+      <c r="O512">
+        <v>27883.1</v>
+      </c>
+      <c r="P512">
+        <v>6</v>
+      </c>
+      <c r="Q512">
+        <v>1.17</v>
+      </c>
+      <c r="R512" t="s">
+        <v>122</v>
+      </c>
+      <c r="S512" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="513" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A513" t="s">
+        <v>113</v>
+      </c>
+      <c r="D513" t="s">
+        <v>50</v>
+      </c>
+      <c r="H513">
+        <v>120</v>
+      </c>
+      <c r="I513" t="s">
+        <v>21</v>
+      </c>
+      <c r="J513">
+        <v>476000</v>
+      </c>
+      <c r="K513">
+        <v>0</v>
+      </c>
+      <c r="L513">
+        <v>0</v>
+      </c>
+      <c r="M513">
+        <v>476000</v>
+      </c>
+      <c r="N513">
+        <v>0</v>
+      </c>
+      <c r="O513">
+        <v>476000</v>
+      </c>
+      <c r="P513">
+        <v>91</v>
+      </c>
+      <c r="Q513">
+        <v>1.32</v>
+      </c>
+      <c r="R513" t="s">
+        <v>122</v>
+      </c>
+      <c r="S513" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="514" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A514" t="s">
+        <v>69</v>
+      </c>
+      <c r="D514" t="s">
+        <v>50</v>
+      </c>
+      <c r="H514">
+        <v>28</v>
+      </c>
+      <c r="I514" t="s">
+        <v>21</v>
+      </c>
+      <c r="J514">
+        <v>140000</v>
+      </c>
+      <c r="K514">
+        <v>0</v>
+      </c>
+      <c r="L514">
+        <v>0</v>
+      </c>
+      <c r="M514">
+        <v>140000</v>
+      </c>
+      <c r="N514">
+        <v>51983.38</v>
+      </c>
+      <c r="O514">
+        <v>88016.62</v>
+      </c>
+      <c r="P514">
+        <v>24</v>
+      </c>
+      <c r="Q514">
+        <v>1.17</v>
+      </c>
+      <c r="R514" t="s">
+        <v>122</v>
+      </c>
+      <c r="S514" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="515" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A515" t="s">
+        <v>70</v>
+      </c>
+      <c r="D515" t="s">
+        <v>71</v>
+      </c>
+      <c r="H515">
+        <v>40</v>
+      </c>
+      <c r="I515" t="s">
+        <v>21</v>
+      </c>
+      <c r="J515">
+        <v>480000</v>
+      </c>
+      <c r="K515">
+        <v>0</v>
+      </c>
+      <c r="L515">
+        <v>0</v>
+      </c>
+      <c r="M515">
+        <v>480000</v>
+      </c>
+      <c r="N515">
+        <v>0</v>
+      </c>
+      <c r="O515">
+        <v>480000</v>
+      </c>
+      <c r="P515">
+        <v>34</v>
+      </c>
+      <c r="Q515">
+        <v>1.18</v>
+      </c>
+      <c r="R515" t="s">
+        <v>122</v>
+      </c>
+      <c r="S515" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="516" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A516" t="s">
+        <v>72</v>
+      </c>
+      <c r="D516" t="s">
+        <v>71</v>
+      </c>
+      <c r="H516">
+        <v>74</v>
+      </c>
+      <c r="I516" t="s">
+        <v>21</v>
+      </c>
+      <c r="J516">
+        <v>886000</v>
+      </c>
+      <c r="K516">
+        <v>0</v>
+      </c>
+      <c r="L516">
+        <v>0</v>
+      </c>
+      <c r="M516">
+        <v>886000</v>
+      </c>
+      <c r="N516">
+        <v>0</v>
+      </c>
+      <c r="O516">
+        <v>886000</v>
+      </c>
+      <c r="P516">
+        <v>72</v>
+      </c>
+      <c r="Q516">
+        <v>1.03</v>
+      </c>
+      <c r="R516" t="s">
+        <v>122</v>
+      </c>
+      <c r="S516" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="517" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A517" t="s">
+        <v>114</v>
+      </c>
+      <c r="D517" t="s">
+        <v>71</v>
+      </c>
+      <c r="H517">
+        <v>28</v>
+      </c>
+      <c r="I517" t="s">
+        <v>21</v>
+      </c>
+      <c r="J517">
+        <v>332000</v>
+      </c>
+      <c r="K517">
+        <v>0</v>
+      </c>
+      <c r="L517">
+        <v>0</v>
+      </c>
+      <c r="M517">
+        <v>332000</v>
+      </c>
+      <c r="N517">
+        <v>0</v>
+      </c>
+      <c r="O517">
+        <v>332000</v>
+      </c>
+      <c r="P517">
+        <v>28</v>
+      </c>
+      <c r="Q517">
+        <v>1</v>
+      </c>
+      <c r="R517" t="s">
+        <v>122</v>
+      </c>
+      <c r="S517" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="518" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A518" t="s">
+        <v>75</v>
+      </c>
+      <c r="D518" t="s">
+        <v>71</v>
+      </c>
+      <c r="H518">
+        <v>45</v>
+      </c>
+      <c r="I518" t="s">
+        <v>21</v>
+      </c>
+      <c r="J518">
+        <v>540000</v>
+      </c>
+      <c r="K518">
+        <v>0</v>
+      </c>
+      <c r="L518">
+        <v>0</v>
+      </c>
+      <c r="M518">
+        <v>540000</v>
+      </c>
+      <c r="N518">
+        <v>0</v>
+      </c>
+      <c r="O518">
+        <v>540000</v>
+      </c>
+      <c r="P518">
+        <v>42</v>
+      </c>
+      <c r="Q518">
+        <v>1.07</v>
+      </c>
+      <c r="R518" t="s">
+        <v>122</v>
+      </c>
+      <c r="S518" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="519" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A519" t="s">
+        <v>115</v>
+      </c>
+      <c r="D519" t="s">
+        <v>71</v>
+      </c>
+      <c r="H519">
+        <v>25</v>
+      </c>
+      <c r="I519" t="s">
+        <v>21</v>
+      </c>
+      <c r="J519">
+        <v>300000</v>
+      </c>
+      <c r="K519">
+        <v>0</v>
+      </c>
+      <c r="L519">
+        <v>0</v>
+      </c>
+      <c r="M519">
+        <v>300000</v>
+      </c>
+      <c r="N519">
+        <v>0</v>
+      </c>
+      <c r="O519">
+        <v>300000</v>
+      </c>
+      <c r="P519">
+        <v>25</v>
+      </c>
+      <c r="Q519">
+        <v>1</v>
+      </c>
+      <c r="R519" t="s">
+        <v>122</v>
+      </c>
+      <c r="S519" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="520" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A520" t="s">
+        <v>77</v>
+      </c>
+      <c r="D520" t="s">
+        <v>71</v>
+      </c>
+      <c r="H520">
+        <v>18</v>
+      </c>
+      <c r="I520" t="s">
+        <v>21</v>
+      </c>
+      <c r="J520">
+        <v>216000</v>
+      </c>
+      <c r="K520">
+        <v>0</v>
+      </c>
+      <c r="L520">
+        <v>0</v>
+      </c>
+      <c r="M520">
+        <v>216000</v>
+      </c>
+      <c r="N520">
+        <v>0</v>
+      </c>
+      <c r="O520">
+        <v>216000</v>
+      </c>
+      <c r="P520">
+        <v>18</v>
+      </c>
+      <c r="Q520">
+        <v>1</v>
+      </c>
+      <c r="R520" t="s">
+        <v>122</v>
+      </c>
+      <c r="S520" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="521" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A521" t="s">
+        <v>117</v>
+      </c>
+      <c r="C521" t="s">
+        <v>72</v>
+      </c>
+      <c r="D521" t="s">
+        <v>71</v>
+      </c>
+      <c r="H521">
+        <v>13</v>
+      </c>
+      <c r="I521" t="s">
+        <v>21</v>
+      </c>
+      <c r="J521">
+        <v>78000</v>
+      </c>
+      <c r="K521">
+        <v>0</v>
+      </c>
+      <c r="L521">
+        <v>0</v>
+      </c>
+      <c r="M521">
+        <v>78000</v>
+      </c>
+      <c r="N521">
+        <v>0</v>
+      </c>
+      <c r="O521">
+        <v>78000</v>
+      </c>
+      <c r="P521">
+        <v>13</v>
+      </c>
+      <c r="Q521">
+        <v>1</v>
+      </c>
+      <c r="R521" t="s">
+        <v>122</v>
+      </c>
+      <c r="S521" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="522" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A522" t="s">
+        <v>117</v>
+      </c>
+      <c r="C522" t="s">
+        <v>124</v>
+      </c>
+      <c r="D522" t="s">
+        <v>71</v>
+      </c>
+      <c r="H522">
+        <v>1</v>
+      </c>
+      <c r="I522" t="s">
+        <v>21</v>
+      </c>
+      <c r="J522">
+        <v>6000</v>
+      </c>
+      <c r="K522">
+        <v>0</v>
+      </c>
+      <c r="L522">
+        <v>0</v>
+      </c>
+      <c r="M522">
+        <v>6000</v>
+      </c>
+      <c r="N522">
+        <v>0</v>
+      </c>
+      <c r="O522">
+        <v>6000</v>
+      </c>
+      <c r="P522">
+        <v>1</v>
+      </c>
+      <c r="Q522">
+        <v>1</v>
+      </c>
+      <c r="R522" t="s">
+        <v>122</v>
+      </c>
+      <c r="S522" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="523" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A523" t="s">
+        <v>117</v>
+      </c>
+      <c r="C523" t="s">
+        <v>114</v>
+      </c>
+      <c r="D523" t="s">
+        <v>71</v>
+      </c>
+      <c r="H523">
+        <v>5</v>
+      </c>
+      <c r="I523" t="s">
+        <v>21</v>
+      </c>
+      <c r="J523">
+        <v>30000</v>
+      </c>
+      <c r="K523">
+        <v>0</v>
+      </c>
+      <c r="L523">
+        <v>0</v>
+      </c>
+      <c r="M523">
+        <v>30000</v>
+      </c>
+      <c r="N523">
+        <v>0</v>
+      </c>
+      <c r="O523">
+        <v>30000</v>
+      </c>
+      <c r="P523">
+        <v>5</v>
+      </c>
+      <c r="Q523">
+        <v>1</v>
+      </c>
+      <c r="R523" t="s">
+        <v>122</v>
+      </c>
+      <c r="S523" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="524" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A524" t="s">
+        <v>117</v>
+      </c>
+      <c r="C524" t="s">
+        <v>118</v>
+      </c>
+      <c r="D524" t="s">
+        <v>71</v>
+      </c>
+      <c r="H524">
+        <v>7</v>
+      </c>
+      <c r="I524" t="s">
+        <v>21</v>
+      </c>
+      <c r="J524">
+        <v>42000</v>
+      </c>
+      <c r="K524">
+        <v>0</v>
+      </c>
+      <c r="L524">
+        <v>0</v>
+      </c>
+      <c r="M524">
+        <v>42000</v>
+      </c>
+      <c r="N524">
+        <v>0</v>
+      </c>
+      <c r="O524">
+        <v>42000</v>
+      </c>
+      <c r="P524">
+        <v>7</v>
+      </c>
+      <c r="Q524">
+        <v>1</v>
+      </c>
+      <c r="R524" t="s">
+        <v>122</v>
+      </c>
+      <c r="S524" t="s">
+        <v>88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>